<commit_message>
Update ASIN planning data March 2026
</commit_message>
<xml_diff>
--- a/data/planning/ASIN Planning file - Mar 2026.xlsx
+++ b/data/planning/ASIN Planning file - Mar 2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\FAstAPI\data\planning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{12EFD83E-AE8D-444C-BBF1-7FE612C5FC87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD45DC82-A345-4FDF-AADB-DB793C0A808B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{A57BF751-5549-4522-BFB9-E6D7D4378C13}"/>
   </bookViews>
@@ -52,18 +52,9 @@
     <t>Model#</t>
   </si>
   <si>
-    <t>March Goal - Projected</t>
-  </si>
-  <si>
     <t>Per Day Goal - Projected</t>
   </si>
   <si>
-    <t>March Goal - Actual</t>
-  </si>
-  <si>
-    <t>March Goal - Actual %</t>
-  </si>
-  <si>
     <t>B0DVC58QPZ</t>
   </si>
   <si>
@@ -649,13 +640,22 @@
     <t>Brand</t>
   </si>
   <si>
-    <t>March Goal</t>
-  </si>
-  <si>
     <t>Per Day Goal</t>
   </si>
   <si>
     <t>Nexlev</t>
+  </si>
+  <si>
+    <t>Mar Goal - Projected</t>
+  </si>
+  <si>
+    <t>Mar Goal - Actual</t>
+  </si>
+  <si>
+    <t>Mar Goal - Actual %</t>
+  </si>
+  <si>
+    <t>Mar Goal</t>
   </si>
 </sst>
 </file>
@@ -2608,31 +2608,31 @@
         <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>5</v>
-      </c>
       <c r="G1" s="3" t="s">
-        <v>6</v>
+        <v>203</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>7</v>
+        <v>204</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B2" t="str">
         <f>_xlfn.XLOOKUP(A2,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Smart Air Purifier </v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E2" s="7">
         <v>305000</v>
@@ -2646,17 +2646,17 @@
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B3" t="str">
         <f>_xlfn.XLOOKUP(A3,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Handheld Garment Steamer </v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E3" s="7">
         <v>447254.23728813563</v>
@@ -2670,17 +2670,17 @@
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B4" t="str">
         <f>_xlfn.XLOOKUP(A4,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Steam Cleaner </v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E4" s="7">
         <v>614194.91525423736</v>
@@ -2694,17 +2694,17 @@
     </row>
     <row r="5" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B5" t="str">
         <f>_xlfn.XLOOKUP(A5,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Portable Cordless Lint Remover </v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E5" s="7">
         <v>64237.288135593226</v>
@@ -2718,17 +2718,17 @@
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B6" t="str">
         <f>_xlfn.XLOOKUP(A6,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Cool Mist Humidifier </v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E6" s="7">
         <v>0</v>
@@ -2742,17 +2742,17 @@
     </row>
     <row r="7" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B7" t="str">
         <f>_xlfn.XLOOKUP(A7,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v>NexLev Steamer For Cold &amp; Cough</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E7" s="7">
         <v>207508.4745762712</v>
@@ -2766,17 +2766,17 @@
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B8" t="str">
         <f>_xlfn.XLOOKUP(A8,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Cool Mist Humidifier </v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E8" s="7">
         <v>198203.38983050847</v>
@@ -2790,17 +2790,17 @@
     </row>
     <row r="9" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B9" t="str">
         <f>_xlfn.XLOOKUP(A9,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v>Nexlev MultiPurpose Electric Food Kettle</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E9" s="7">
         <v>162610.16949152542</v>
@@ -2814,17 +2814,17 @@
     </row>
     <row r="10" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B10" t="str">
         <f>_xlfn.XLOOKUP(A10,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v>nexlev Ionic 3 In 1 Hot Air Brush</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E10" s="7">
         <v>0</v>
@@ -2838,17 +2838,17 @@
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B11" t="str">
         <f>_xlfn.XLOOKUP(A11,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Mattress, Sofa &amp; Carpet Vacuum Cleaner </v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E11" s="7">
         <v>786169.49152542371</v>
@@ -2862,17 +2862,17 @@
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B12" t="str">
         <f>_xlfn.XLOOKUP(A12,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Foldable Garment Steamer for Home &amp; Travel </v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E12" s="7">
         <v>235042.37288135596</v>
@@ -2886,17 +2886,17 @@
     </row>
     <row r="13" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B13" t="str">
         <f>_xlfn.XLOOKUP(A13,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v>Nexlev Multi Purpose Electric Food Kettle</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="E13" s="7">
         <v>148220.33898305087</v>
@@ -2910,17 +2910,17 @@
     </row>
     <row r="14" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B14" t="str">
         <f>_xlfn.XLOOKUP(A14,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Blackhead &amp; Whitehead Remover Tool </v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E14" s="7">
         <v>203262.7118644068</v>
@@ -2934,17 +2934,17 @@
     </row>
     <row r="15" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B15" t="str">
         <f>_xlfn.XLOOKUP(A15,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev LED Phototherapy comb </v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E15" s="7">
         <v>241398.30508474578</v>
@@ -2958,17 +2958,17 @@
     </row>
     <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B16" t="str">
         <f>_xlfn.XLOOKUP(A16,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Calf Massager </v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="E16" s="7">
         <v>379525.42372881359</v>
@@ -2982,17 +2982,17 @@
     </row>
     <row r="17" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B17" t="str">
         <f>_xlfn.XLOOKUP(A17,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev LED Therapy Oil Applicator </v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E17" s="7">
         <v>139703.38983050847</v>
@@ -3006,17 +3006,17 @@
     </row>
     <row r="18" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B18" t="str">
         <f>_xlfn.XLOOKUP(A18,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v>NexLev Cordless Electric Heating Pad</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E18" s="7">
         <v>0</v>
@@ -3030,17 +3030,17 @@
     </row>
     <row r="19" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B19" t="str">
         <f>_xlfn.XLOOKUP(A19,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Steam Cleaner </v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="E19" s="7">
         <v>1186101.6949152544</v>
@@ -3054,17 +3054,17 @@
     </row>
     <row r="20" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B20" t="str">
         <f>_xlfn.XLOOKUP(A20,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Portable Blender for Smoothies Milkshakes Crushing Ice Juices </v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="E20" s="7">
         <v>149084.74576271189</v>
@@ -3078,17 +3078,17 @@
     </row>
     <row r="21" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B21" t="str">
         <f>_xlfn.XLOOKUP(A21,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Stand Mixer </v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E21" s="7">
         <v>477033.89830508479</v>
@@ -3102,17 +3102,17 @@
     </row>
     <row r="22" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B22" t="str">
         <f>_xlfn.XLOOKUP(A22,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Mini Electric Chopper </v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="E22" s="7">
         <v>0</v>
@@ -3126,17 +3126,17 @@
     </row>
     <row r="23" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B23" t="str">
         <f>_xlfn.XLOOKUP(A23,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">Nexlev SWIPE Steam Cleaner </v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E23" s="7">
         <v>0</v>
@@ -3150,17 +3150,17 @@
     </row>
     <row r="24" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B24" t="str">
         <f>_xlfn.XLOOKUP(A24,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Rechargeable Lint Remover </v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E24" s="7">
         <v>228661.01694915254</v>
@@ -3174,17 +3174,17 @@
     </row>
     <row r="25" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B25" t="str">
         <f>_xlfn.XLOOKUP(A25,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Ionic Cordless Hair Straightener Brush </v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="E25" s="7">
         <v>290559.32203389832</v>
@@ -3198,17 +3198,17 @@
     </row>
     <row r="26" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B26" t="str">
         <f>_xlfn.XLOOKUP(A26,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v>nexlev Ionic Volumizer</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="E26" s="7">
         <v>0</v>
@@ -3222,17 +3222,17 @@
     </row>
     <row r="27" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B27" t="str">
         <f>_xlfn.XLOOKUP(A27,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v>NexLev Oil Applicator Comb</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="E27" s="7">
         <v>220254.2372881356</v>
@@ -3246,17 +3246,17 @@
     </row>
     <row r="28" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B28" t="str">
         <f>_xlfn.XLOOKUP(A28,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Smart Electric Toothbrush for Adults </v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E28" s="7">
         <v>45610.169491525427</v>
@@ -3270,17 +3270,17 @@
     </row>
     <row r="29" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B29" t="str">
         <f>_xlfn.XLOOKUP(A29,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Smart Electric Toothbrush for Adults </v>
       </c>
       <c r="C29" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D29" s="6" t="s">
         <v>68</v>
-      </c>
-      <c r="D29" s="6" t="s">
-        <v>71</v>
       </c>
       <c r="E29" s="7">
         <v>30406.77966101695</v>
@@ -3294,13 +3294,13 @@
     </row>
     <row r="30" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="E30" s="7">
         <v>0</v>
@@ -3314,17 +3314,17 @@
     </row>
     <row r="31" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B31" t="str">
         <f>_xlfn.XLOOKUP(A31,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Air Purifier for Living Room </v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E31" s="7">
         <v>0</v>
@@ -3338,17 +3338,17 @@
     </row>
     <row r="32" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B32" t="str">
         <f>_xlfn.XLOOKUP(A32,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v>NexLev Portable Tyre Inflator for Car, Bike, Cycle</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E32" s="7">
         <v>0</v>
@@ -3362,17 +3362,17 @@
     </row>
     <row r="33" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B33" t="str">
         <f>_xlfn.XLOOKUP(A33,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v>NexLev Ionic Hair Straightener Brush for Woman</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="E33" s="7">
         <v>128745.76271186442</v>
@@ -3386,17 +3386,17 @@
     </row>
     <row r="34" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B34" t="str">
         <f>_xlfn.XLOOKUP(A34,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Rechargeable Milk Frother &amp; Coffee Whisker </v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="E34" s="7">
         <v>0</v>
@@ -3410,17 +3410,17 @@
     </row>
     <row r="35" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B35" t="str">
         <f>_xlfn.XLOOKUP(A35,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Rechargeable Lint Remover </v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="E35" s="7">
         <v>45711.864406779663</v>
@@ -3434,17 +3434,17 @@
     </row>
     <row r="36" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B36" t="str">
         <f>_xlfn.XLOOKUP(A36,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Ionic Hot Air Brush </v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="E36" s="7">
         <v>0</v>
@@ -3458,13 +3458,13 @@
     </row>
     <row r="37" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="E37" s="7">
         <v>0</v>
@@ -3478,17 +3478,17 @@
     </row>
     <row r="38" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B38" t="str">
         <f>_xlfn.XLOOKUP(A38,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Foot Callus Remover </v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E38" s="7">
         <v>47389.830508474581</v>
@@ -3502,17 +3502,17 @@
     </row>
     <row r="39" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B39" t="str">
         <f>_xlfn.XLOOKUP(A39,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v>NexLev Intimate Trimmer for Men</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="E39" s="7">
         <v>0</v>
@@ -3526,17 +3526,17 @@
     </row>
     <row r="40" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B40" t="str">
         <f>_xlfn.XLOOKUP(A40,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">Nexlev Oscillating Electric Toothbrush </v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="E40" s="7">
         <v>31754.237288135595</v>
@@ -3550,17 +3550,17 @@
     </row>
     <row r="41" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B41" t="str">
         <f>_xlfn.XLOOKUP(A41,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v>NexLev Cordless Electric Heating Pad</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="E41" s="7">
         <v>68593.220338983054</v>
@@ -3574,17 +3574,17 @@
     </row>
     <row r="42" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B42" t="str">
         <f>_xlfn.XLOOKUP(A42,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v>Nexlev Rechargeable Electric Toothbrush</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="E42" s="7">
         <v>38084.745762711864</v>
@@ -3598,17 +3598,17 @@
     </row>
     <row r="43" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B43" t="str">
         <f>_xlfn.XLOOKUP(A43,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v>Nexlev Rechargeable Electric Toothbrush</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="E43" s="7">
         <v>63474.576271186445</v>
@@ -3622,17 +3622,17 @@
     </row>
     <row r="44" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B44" t="str">
         <f>_xlfn.XLOOKUP(A44,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">Nexlev Skin Scrubber </v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="E44" s="7">
         <v>43194.91525423729</v>
@@ -3646,17 +3646,17 @@
     </row>
     <row r="45" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B45" t="str">
         <f>_xlfn.XLOOKUP(A45,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v>NexLev IONIC Volumizer + Straightening Brush</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="E45" s="7">
         <v>0</v>
@@ -3670,17 +3670,17 @@
     </row>
     <row r="46" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B46" t="str">
         <f>_xlfn.XLOOKUP(A46,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v>NexLev Beard Trimmer</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="E46" s="7">
         <v>0</v>
@@ -3694,17 +3694,17 @@
     </row>
     <row r="47" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="4" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B47" t="str">
         <f>_xlfn.XLOOKUP(A47,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v>Nexlev Hair Styling Straightener &amp; Curler</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="E47" s="7">
         <v>0</v>
@@ -3718,17 +3718,17 @@
     </row>
     <row r="48" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="4" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B48" t="str">
         <f>_xlfn.XLOOKUP(A48,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v>NexLev Calf Massager Pro</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="E48" s="7">
         <v>35587.288135593219</v>
@@ -3742,17 +3742,17 @@
     </row>
     <row r="49" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="4" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B49" t="str">
         <f>_xlfn.XLOOKUP(A49,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">Nexlev Skin Lift Device </v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="E49" s="7">
         <v>50813.5593220339</v>
@@ -3766,17 +3766,17 @@
     </row>
     <row r="50" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="4" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B50" t="str">
         <f>_xlfn.XLOOKUP(A50,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Massage Gun </v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="E50" s="7">
         <v>0</v>
@@ -3790,17 +3790,17 @@
     </row>
     <row r="51" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="4" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B51" t="str">
         <f>_xlfn.XLOOKUP(A51,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Body &amp; Intimate Trimmer for Men </v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="E51" s="7">
         <v>0</v>
@@ -3814,17 +3814,17 @@
     </row>
     <row r="52" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="4" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B52" t="str">
         <f>_xlfn.XLOOKUP(A52,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">Nexlev Tyre Inflator for Car </v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="E52" s="7">
         <v>0</v>
@@ -3838,17 +3838,17 @@
     </row>
     <row r="53" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="4" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B53" t="str">
         <f>_xlfn.XLOOKUP(A53,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">Nexlev Just Style Pro Hair Dryer </v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="E53" s="7">
         <v>0</v>
@@ -3862,17 +3862,17 @@
     </row>
     <row r="54" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="4" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B54" t="str">
         <f>_xlfn.XLOOKUP(A54,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev All in One Body Trimmer for Men </v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="E54" s="7">
         <v>0</v>
@@ -3886,17 +3886,17 @@
     </row>
     <row r="55" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="4" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B55" t="str">
         <f>_xlfn.XLOOKUP(A55,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Massage Gun </v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="E55" s="7">
         <v>0</v>
@@ -3910,17 +3910,17 @@
     </row>
     <row r="56" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="4" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B56" t="str">
         <f>_xlfn.XLOOKUP(A56,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev 2 in 1 Handheld &amp; Stick Vacuum Cleaner </v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="E56" s="7">
         <v>266822.03389830509</v>
@@ -3934,17 +3934,17 @@
     </row>
     <row r="57" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="4" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B57" t="str">
         <f>_xlfn.XLOOKUP(A57,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev 1500W Electric Water Kettle </v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="E57" s="7">
         <v>0</v>
@@ -3958,17 +3958,17 @@
     </row>
     <row r="58" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="4" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B58" t="str">
         <f>_xlfn.XLOOKUP(A58,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v>NexLev Cordless Vacuum Cleaner</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E58" s="7">
         <v>0</v>
@@ -3982,17 +3982,17 @@
     </row>
     <row r="59" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="4" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B59" t="str">
         <f>_xlfn.XLOOKUP(A59,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v>Nexlev Electric Toothbrush</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="E59" s="7">
         <v>0</v>
@@ -4006,17 +4006,17 @@
     </row>
     <row r="60" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="4" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B60" t="str">
         <f>_xlfn.XLOOKUP(A60,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v>nexlev Cordless Wet &amp; Dry Vacuum Cleaner</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="E60" s="7">
         <v>71152.542372881362</v>
@@ -4030,17 +4030,17 @@
     </row>
     <row r="61" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="4" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="B61" t="str">
         <f>_xlfn.XLOOKUP(A61,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">nexlev Cordless Vacuum Cleaner &amp; Blower </v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="E61" s="7">
         <v>0</v>
@@ -4054,17 +4054,17 @@
     </row>
     <row r="62" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="4" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B62" t="str">
         <f>_xlfn.XLOOKUP(A62,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v>Nexlev Cordless &amp; Corded Tyre Inflator</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="E62" s="7">
         <v>0</v>
@@ -4078,17 +4078,17 @@
     </row>
     <row r="63" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="4" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="B63" t="str">
         <f>_xlfn.XLOOKUP(A63,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v>nexlev Cordless Electric Car Vacuum Cleaner VacuSafe</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="E63" s="7">
         <v>0</v>
@@ -4102,17 +4102,17 @@
     </row>
     <row r="64" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="4" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B64" t="str">
         <f>_xlfn.XLOOKUP(A64,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">nexlev Travel Neck Pillow </v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="E64" s="7">
         <v>0</v>
@@ -4126,17 +4126,17 @@
     </row>
     <row r="65" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="4" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="B65" t="str">
         <f>_xlfn.XLOOKUP(A65,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">nexlev Travel Neck Pillow </v>
       </c>
       <c r="C65" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="D65" s="6" t="s">
         <v>143</v>
-      </c>
-      <c r="D65" s="6" t="s">
-        <v>146</v>
       </c>
       <c r="E65" s="7">
         <v>0</v>
@@ -4150,13 +4150,13 @@
     </row>
     <row r="66" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="4" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="E66" s="7">
         <v>0</v>
@@ -4170,17 +4170,17 @@
     </row>
     <row r="67" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="4" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B67" t="str">
         <f>_xlfn.XLOOKUP(A67,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v>NexLev Mattress, Sofa, Carpet &amp; Car Seat Vacuum Cleaner</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="E67" s="7">
         <v>518491.52542372886</v>
@@ -4194,13 +4194,13 @@
     </row>
     <row r="68" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="4" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="E68" s="7">
         <v>0</v>
@@ -4214,17 +4214,17 @@
     </row>
     <row r="69" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="4" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="B69" t="str">
         <f>_xlfn.XLOOKUP(A69,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Travel Neck Pillow </v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="E69" s="7">
         <v>0</v>
@@ -4238,13 +4238,13 @@
     </row>
     <row r="70" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="4" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C70" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="E70" s="7">
         <v>0</v>
@@ -4258,17 +4258,17 @@
     </row>
     <row r="71" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="4" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B71" t="str">
         <f>_xlfn.XLOOKUP(A71,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v>NexLev Spin Scrubber</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D71" s="6" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="E71" s="7">
         <v>0</v>
@@ -4282,17 +4282,17 @@
     </row>
     <row r="72" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="4" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B72" t="str">
         <f>_xlfn.XLOOKUP(A72,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Travel Neck Pillow </v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E72" s="7">
         <v>0</v>
@@ -4306,17 +4306,17 @@
     </row>
     <row r="73" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="4" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="B73" t="str">
         <f>_xlfn.XLOOKUP(A73,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v>NexLev 10 in 1 Steam Cleaner &amp; Mop</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="E73" s="7">
         <v>762584.74576271186</v>
@@ -4330,17 +4330,17 @@
     </row>
     <row r="74" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="4" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B74" t="str">
         <f>_xlfn.XLOOKUP(A74,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v>NexLev 2 in 1 Nose, Ear &amp; Body Trimmer for Men</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E74" s="7">
         <v>0</v>
@@ -4354,17 +4354,17 @@
     </row>
     <row r="75" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="4" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="B75" t="str">
         <f>_xlfn.XLOOKUP(A75,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Steam Mop </v>
       </c>
       <c r="C75" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="E75" s="7">
         <v>0</v>
@@ -4378,17 +4378,17 @@
     </row>
     <row r="76" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="4" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="B76" t="str">
         <f>_xlfn.XLOOKUP(A76,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Drip Coffee Maker </v>
       </c>
       <c r="C76" s="5" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D76" s="6" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="E76" s="7">
         <v>0</v>
@@ -4402,13 +4402,13 @@
     </row>
     <row r="77" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="4" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C77" s="5" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D77" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="E77" s="7">
         <v>0</v>
@@ -4422,17 +4422,17 @@
     </row>
     <row r="78" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="4" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="B78" t="str">
         <f>_xlfn.XLOOKUP(A78,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Handheld Garment Steamer </v>
       </c>
       <c r="C78" s="5" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D78" s="6" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E78" s="7">
         <v>0</v>
@@ -4446,17 +4446,17 @@
     </row>
     <row r="79" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="4" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="B79" t="str">
         <f>_xlfn.XLOOKUP(A79,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">Nexlev Splash Pet Water Fountain with LED Light </v>
       </c>
       <c r="C79" s="5" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="D79" s="6" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="E79" s="7">
         <v>0</v>
@@ -4470,17 +4470,17 @@
     </row>
     <row r="80" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="4" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B80" t="str">
         <f>_xlfn.XLOOKUP(A80,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Massage Gun </v>
       </c>
       <c r="C80" s="5" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D80" s="6" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="E80" s="7">
         <v>0</v>
@@ -4494,17 +4494,17 @@
     </row>
     <row r="81" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="4" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B81" t="str">
         <f>_xlfn.XLOOKUP(A81,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v>Nexlev Rechargeable Electric Toothbrush</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D81" s="6" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="E81" s="7">
         <v>38084.745762711864</v>
@@ -4518,17 +4518,17 @@
     </row>
     <row r="82" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="4" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="B82" t="str">
         <f>_xlfn.XLOOKUP(A82,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v>Nexlev Hair Styling Straightener &amp; Curler</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D82" s="6" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="E82" s="7">
         <v>0</v>
@@ -4542,17 +4542,17 @@
     </row>
     <row r="83" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="4" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="B83" t="str">
         <f>_xlfn.XLOOKUP(A83,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Spin Scrubber with Soap Spray </v>
       </c>
       <c r="C83" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D83" s="6" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="E83" s="7">
         <v>0</v>
@@ -4566,17 +4566,17 @@
     </row>
     <row r="84" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="4" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="B84" t="str">
         <f>_xlfn.XLOOKUP(A84,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v>Nexlev Portable Sewing Machine</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D84" s="6" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="E84" s="7">
         <v>0</v>
@@ -4590,13 +4590,13 @@
     </row>
     <row r="85" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A85" s="4" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="C85" s="5" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D85" s="6" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="E85" s="7">
         <v>0</v>
@@ -4610,17 +4610,17 @@
     </row>
     <row r="86" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="4" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="B86" t="str">
         <f>_xlfn.XLOOKUP(A86,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev 6-in-1 trimmer </v>
       </c>
       <c r="C86" s="5" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D86" s="6" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="E86" s="7">
         <v>0</v>
@@ -4634,17 +4634,17 @@
     </row>
     <row r="87" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="4" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B87" t="str">
         <f>_xlfn.XLOOKUP(A87,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Steam Cleaner </v>
       </c>
       <c r="C87" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D87" s="6" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="E87" s="7">
         <v>0</v>
@@ -4658,17 +4658,17 @@
     </row>
     <row r="88" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="4" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="B88" t="str">
         <f>_xlfn.XLOOKUP(A88,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Scalp Massager for Stress Relief </v>
       </c>
       <c r="C88" s="5" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D88" s="6" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="E88" s="7">
         <v>0</v>
@@ -4682,13 +4682,13 @@
     </row>
     <row r="89" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="4" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="C89" s="5" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D89" s="6" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="E89" s="7">
         <v>0</v>
@@ -4702,17 +4702,17 @@
     </row>
     <row r="90" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="4" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="B90" t="str">
         <f>_xlfn.XLOOKUP(A90,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev 6-in-1 trimmer </v>
       </c>
       <c r="C90" s="5" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D90" s="6" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="E90" s="7">
         <v>0</v>
@@ -4726,17 +4726,17 @@
     </row>
     <row r="91" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A91" s="9" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="B91" t="str">
         <f>_xlfn.XLOOKUP(A91,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Calf Massager </v>
       </c>
       <c r="C91" s="5" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D91" s="8" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="E91" s="7">
         <v>84728.813559322036</v>
@@ -4750,17 +4750,17 @@
     </row>
     <row r="92" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="4" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="B92" t="str">
         <f>_xlfn.XLOOKUP(A92,[1]Sheet1!$C:$C,[1]Sheet1!$E:$E)</f>
         <v xml:space="preserve">NexLev Dehumidifier for Room Moisture Absorption </v>
       </c>
       <c r="C92" s="5" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D92" s="8" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="E92" s="7">
         <v>67779.661016949161</v>
@@ -4791,24 +4791,24 @@
   <sheetData>
     <row r="1" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="B1" s="10" t="s">
         <v>2</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C2">
         <v>570983.05084745772</v>
@@ -4819,10 +4819,10 @@
     </row>
     <row r="3" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -4833,10 +4833,10 @@
     </row>
     <row r="4" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C4">
         <v>4205516.9491525423</v>
@@ -4847,10 +4847,10 @@
     </row>
     <row r="5" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C5">
         <v>568434.74576271186</v>
@@ -4861,10 +4861,10 @@
     </row>
     <row r="6" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C6">
         <v>1020906.779661017</v>
@@ -4875,10 +4875,10 @@
     </row>
     <row r="7" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C7">
         <v>1020661.0169491526</v>
@@ -4889,10 +4889,10 @@
     </row>
     <row r="8" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C8">
         <v>936949.15254237293</v>
@@ -4903,10 +4903,10 @@
     </row>
     <row r="9" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C9">
         <v>247415.25423728814</v>
@@ -4917,10 +4917,10 @@
     </row>
     <row r="10" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -4931,10 +4931,10 @@
     </row>
     <row r="11" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C11">
         <v>552169.49152542383</v>
@@ -4945,10 +4945,10 @@
     </row>
     <row r="12" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="C12">
         <v>0</v>
@@ -4959,10 +4959,10 @@
     </row>
     <row r="13" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C13">
         <v>0</v>

</xml_diff>